<commit_message>
chore: nightly sync from Google Sheets [2026-03-08 09:37 UTC]
</commit_message>
<xml_diff>
--- a/data/Sheet1.xlsx
+++ b/data/Sheet1.xlsx
@@ -413,48 +413,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>S.NO</t>
+          <t>product_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Product Name</t>
+          <t>product_name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>category</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Dimensions ( L X B X H )</t>
+          <t>size</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>color</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>price (â¹)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Product Image</t>
+          <t>image_url</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BAG001</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>Tote Bag</t>
@@ -462,17 +476,37 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+          <t>Tote</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MULTI</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1200</v>
+      </c>
       <c r="G2" t="inlineStr"/>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>A stylish everyday Tote bag to carry your essentials, available in custom color in medium and large sizes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BAG001</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -481,176 +515,380 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Tote</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>26 cm X 28 cm x 10 cm</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MULTI</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1400</v>
+      </c>
       <c r="G3" t="inlineStr"/>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>A stylish everyday Tote bag to carry your essentials, available in custom color in medium and large sizes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BAG002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Clutch Koodai</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Clutch</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">33 cm X 31 cm X 12 cm </t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MULTI</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>700</v>
+      </c>
       <c r="G4" t="inlineStr"/>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>An effortless style statement to complete your look</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BAG002</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Clutch Koodai</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Clutch</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>36 cm X 34 cm X 14 cm</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>MULTI</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1000</v>
+      </c>
       <c r="G5" t="inlineStr"/>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>An effortless style statement to complete your look</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAG002 </t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Clutch </t>
+          <t>Clutch Koodai</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+          <t>Clutch</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>MULTI</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>700</v>
+      </c>
       <c r="G6" t="inlineStr"/>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>An effortless style statement to complete your look</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BAG003</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sling with chain</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+          <t>Sling</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>MULTI</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>900</v>
+      </c>
       <c r="G7" t="inlineStr"/>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>A timeless style statement with elegant handle</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BAG003</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sling with chain</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+          <t>Sling</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MULTI</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1200</v>
+      </c>
       <c r="G8" t="inlineStr"/>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>A timeless style statement with elegant handle</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>7</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BAG003</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Sling with chain</t>
+          <t>Sling with leather</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+          <t>Sling</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MULTI</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1100</v>
+      </c>
       <c r="G9" t="inlineStr"/>
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>A timeless style statement with elegant handle</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BAG003</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sling with leather</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+          <t>Sling</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>MULTI</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1400</v>
+      </c>
       <c r="G10" t="inlineStr"/>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>A timeless style statement with elegant handle</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>9</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BAG004</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sling with handle</t>
+          <t>Basket Koodai</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
+          <t>Basket</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="n">
+        <v>650</v>
+      </c>
       <c r="G11" t="inlineStr"/>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BAG004</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Basket Koodai</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
+          <t>Basket</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="n">
+        <v>850</v>
+      </c>
       <c r="G12" t="inlineStr"/>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>11</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BAG004</t>
+        </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -659,47 +897,103 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>Basket</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="n">
+        <v>1100</v>
+      </c>
       <c r="G13" t="inlineStr"/>
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BAG005</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Wooden handle Koodai</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
+          <t>Wooden</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="n">
+        <v>750</v>
+      </c>
       <c r="G14" t="inlineStr"/>
+      <c r="H14" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BAG005</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Wooden handle Koodai</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>Wooden</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="n">
+        <v>1000</v>
+      </c>
       <c r="G15" t="inlineStr"/>
+      <c r="H15" t="b">
+        <v>1</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>14</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BAG005</t>
+        </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -708,199 +1002,272 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>Wooden</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="n">
+        <v>1400</v>
+      </c>
       <c r="G16" t="inlineStr"/>
+      <c r="H16" t="b">
+        <v>1</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BAG005</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Kai Koodai</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>Wooden</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="n">
+        <v>750</v>
+      </c>
       <c r="G17" t="inlineStr"/>
+      <c r="H17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BAG005</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Kai Koodai</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>Wooden</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="n">
+        <v>950</v>
+      </c>
       <c r="G18" t="inlineStr"/>
+      <c r="H18" t="b">
+        <v>1</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>17</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BAG005</t>
+        </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Kai Koodai</t>
+          <t>Eye handle Koodai</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Wooden</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>21 x 21 x 8</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="n">
+        <v>850</v>
+      </c>
       <c r="G19" t="inlineStr"/>
+      <c r="H19" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Ultra stylish bag, a perfect head turner!</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BAG005</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Eye handle Koodai</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Wooden</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>28 x 28 x 10</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="n">
+        <v>1100</v>
+      </c>
       <c r="G20" t="inlineStr"/>
+      <c r="H20" t="b">
+        <v>1</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Ultra stylish bag, a perfect head turner!</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BAG005</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Eye handle Koodai</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Wooden</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>30 x 30 x 11</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="n">
+        <v>1400</v>
+      </c>
       <c r="G21" t="inlineStr"/>
+      <c r="H21" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Ultra stylish bag, a perfect head turner!</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
-        <v>20</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BAG005</t>
+        </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Eye handle Koodai</t>
+          <t>Cute Pooja Koodai</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>21 x 21 x 8</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="n">
+        <v>850</v>
+      </c>
       <c r="G22" t="inlineStr"/>
+      <c r="H22" t="b">
+        <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BAG005</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Cute Pooja Koodai</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>28 x 28 x 10</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="n">
+        <v>1000</v>
+      </c>
       <c r="G23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>30 x 30 x 11</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Cute Pooja Basket</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="H23" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: nightly sync from Google Sheets [2026-03-08 10:55 UTC]
</commit_message>
<xml_diff>
--- a/data/Sheet1.xlsx
+++ b/data/Sheet1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,15 +449,10 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>image_url</t>
+          <t>in_stock</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
-        <is>
-          <t>in_stock</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -492,11 +487,10 @@
       <c r="F2" t="n">
         <v>1200</v>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>A stylish everyday Tote bag to carry your essentials, available in custom color in medium and large sizes</t>
         </is>
@@ -531,11 +525,10 @@
       <c r="F3" t="n">
         <v>1400</v>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="b">
+      <c r="G3" t="b">
         <v>0</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>A stylish everyday Tote bag to carry your essentials, available in custom color in medium and large sizes</t>
         </is>
@@ -570,11 +563,10 @@
       <c r="F4" t="n">
         <v>700</v>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>An effortless style statement to complete your look</t>
         </is>
@@ -609,11 +601,10 @@
       <c r="F5" t="n">
         <v>1000</v>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>An effortless style statement to complete your look</t>
         </is>
@@ -648,11 +639,10 @@
       <c r="F6" t="n">
         <v>700</v>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>An effortless style statement to complete your look</t>
         </is>
@@ -687,11 +677,10 @@
       <c r="F7" t="n">
         <v>900</v>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>A timeless style statement with elegant handle</t>
         </is>
@@ -726,11 +715,10 @@
       <c r="F8" t="n">
         <v>1200</v>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>A timeless style statement with elegant handle</t>
         </is>
@@ -765,11 +753,10 @@
       <c r="F9" t="n">
         <v>1100</v>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" t="inlineStr">
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>A timeless style statement with elegant handle</t>
         </is>
@@ -804,11 +791,10 @@
       <c r="F10" t="n">
         <v>1400</v>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>A timeless style statement with elegant handle</t>
         </is>
@@ -839,11 +825,10 @@
       <c r="F11" t="n">
         <v>650</v>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" t="inlineStr">
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>Your everyday travel buddy, for that sturdy yet cute look</t>
         </is>
@@ -874,11 +859,10 @@
       <c r="F12" t="n">
         <v>850</v>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" t="inlineStr">
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>Your everyday travel buddy, for that sturdy yet cute look</t>
         </is>
@@ -909,11 +893,10 @@
       <c r="F13" t="n">
         <v>1100</v>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I13" t="inlineStr">
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>Your everyday travel buddy, for that sturdy yet cute look</t>
         </is>
@@ -944,11 +927,10 @@
       <c r="F14" t="n">
         <v>750</v>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="b">
-        <v>1</v>
-      </c>
-      <c r="I14" t="inlineStr">
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
         </is>
@@ -979,11 +961,10 @@
       <c r="F15" t="n">
         <v>1000</v>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="b">
-        <v>1</v>
-      </c>
-      <c r="I15" t="inlineStr">
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
         </is>
@@ -1014,11 +995,10 @@
       <c r="F16" t="n">
         <v>1400</v>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="b">
-        <v>1</v>
-      </c>
-      <c r="I16" t="inlineStr">
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
         </is>
@@ -1049,11 +1029,10 @@
       <c r="F17" t="n">
         <v>750</v>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="b">
-        <v>1</v>
-      </c>
-      <c r="I17" t="inlineStr">
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
         </is>
@@ -1084,11 +1063,10 @@
       <c r="F18" t="n">
         <v>950</v>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="b">
-        <v>1</v>
-      </c>
-      <c r="I18" t="inlineStr">
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
         </is>
@@ -1119,11 +1097,10 @@
       <c r="F19" t="n">
         <v>850</v>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="b">
-        <v>1</v>
-      </c>
-      <c r="I19" t="inlineStr">
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>Ultra stylish bag, a perfect head turner!</t>
         </is>
@@ -1154,11 +1131,10 @@
       <c r="F20" t="n">
         <v>1100</v>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="b">
-        <v>1</v>
-      </c>
-      <c r="I20" t="inlineStr">
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>Ultra stylish bag, a perfect head turner!</t>
         </is>
@@ -1189,11 +1165,10 @@
       <c r="F21" t="n">
         <v>1400</v>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="b">
-        <v>1</v>
-      </c>
-      <c r="I21" t="inlineStr">
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>Ultra stylish bag, a perfect head turner!</t>
         </is>
@@ -1224,11 +1199,10 @@
       <c r="F22" t="n">
         <v>850</v>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="b">
-        <v>1</v>
-      </c>
-      <c r="I22" t="inlineStr">
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
         </is>
@@ -1259,11 +1233,10 @@
       <c r="F23" t="n">
         <v>1000</v>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="b">
-        <v>1</v>
-      </c>
-      <c r="I23" t="inlineStr">
+      <c r="G23" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
         </is>

</xml_diff>

<commit_message>
chore: nightly sync from Google Sheets [2026-03-08 12:56 UTC]
</commit_message>
<xml_diff>
--- a/data/Sheet1.xlsx
+++ b/data/Sheet1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -613,17 +613,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">BAG002 </t>
+          <t>BAG003</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Clutch Koodai</t>
+          <t>Sling with chain</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Clutch</t>
+          <t>Sling</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -637,14 +637,14 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>700</v>
+        <v>900</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>An effortless style statement to complete your look</t>
+          <t>A timeless style statement with elegant handle</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>900</v>
+        <v>1200</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
@@ -694,7 +694,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sling with chain</t>
+          <t>Sling with leather</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="G8" t="b">
         <v>1</v>
@@ -742,7 +742,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1100</v>
+        <v>1400</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
@@ -765,38 +765,34 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BAG003</t>
+          <t>BAG004</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sling with leather</t>
+          <t>Basket Koodai</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sling</t>
+          <t>Basket</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>MULTI</t>
-        </is>
-      </c>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>1400</v>
+        <v>650</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>A timeless style statement with elegant handle</t>
+          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
         </is>
       </c>
     </row>
@@ -818,12 +814,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>650</v>
+        <v>850</v>
       </c>
       <c r="G11" t="b">
         <v>1</v>
@@ -852,12 +848,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>850</v>
+        <v>1100</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
@@ -871,34 +867,34 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BAG004</t>
+          <t>BAG005</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Basket Koodai</t>
+          <t>Wooden handle Koodai</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Basket</t>
+          <t>Wooden</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>1100</v>
+        <v>750</v>
       </c>
       <c r="G13" t="b">
         <v>1</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
+          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
         </is>
       </c>
     </row>
@@ -920,12 +916,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="G14" t="b">
         <v>1</v>
@@ -954,12 +950,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>1000</v>
+        <v>1400</v>
       </c>
       <c r="G15" t="b">
         <v>1</v>
@@ -978,7 +974,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Wooden handle Koodai</t>
+          <t>Kai Koodai</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -988,19 +984,19 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>1400</v>
+        <v>750</v>
       </c>
       <c r="G16" t="b">
         <v>1</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
+          <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1018,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>750</v>
+        <v>950</v>
       </c>
       <c r="G17" t="b">
         <v>1</v>
@@ -1046,7 +1042,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Kai Koodai</t>
+          <t>Eye handle Koodai</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1056,19 +1052,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>950</v>
+        <v>850</v>
       </c>
       <c r="G18" t="b">
         <v>1</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
+          <t>Ultra stylish bag, a perfect head turner!</t>
         </is>
       </c>
     </row>
@@ -1090,12 +1086,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>850</v>
+        <v>1100</v>
       </c>
       <c r="G19" t="b">
         <v>1</v>
@@ -1124,12 +1120,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>1100</v>
+        <v>1400</v>
       </c>
       <c r="G20" t="b">
         <v>1</v>
@@ -1148,29 +1144,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Eye handle Koodai</t>
+          <t>Cute Pooja Koodai</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Pooja</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
-        <v>1400</v>
+        <v>850</v>
       </c>
       <c r="G21" t="b">
         <v>1</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Ultra stylish bag, a perfect head turner!</t>
+          <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
         </is>
       </c>
     </row>
@@ -1192,51 +1188,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>850</v>
+        <v>1000</v>
       </c>
       <c r="G22" t="b">
         <v>1</v>
       </c>
       <c r="H22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>BAG005</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Cute Pooja Koodai</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Pooja</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G23" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" t="inlineStr">
         <is>
           <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
         </is>

</xml_diff>

<commit_message>
chore: nightly sync from Google Sheets [2026-03-09 03:44 UTC]
</commit_message>
<xml_diff>
--- a/data/Sheet1.xlsx
+++ b/data/Sheet1.xlsx
@@ -1139,7 +1139,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG006</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pooja</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1173,7 +1173,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG006</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">

</xml_diff>

<commit_message>
chore: nightly sync from Google Sheets [2026-03-09 07:13 UTC]
</commit_message>
<xml_diff>
--- a/data/Sheet1.xlsx
+++ b/data/Sheet1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,10 +449,15 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>image_url</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>in_stock</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -487,10 +492,15 @@
       <c r="F2" t="n">
         <v>1200</v>
       </c>
-      <c r="G2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Biscuit Knot Tote.jpg, White Tote Bag.jpg, Dimensions Chart.png</t>
+        </is>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>A stylish everyday Tote bag to carry your essentials, available in custom color in medium and large sizes</t>
         </is>
@@ -525,10 +535,11 @@
       <c r="F3" t="n">
         <v>1400</v>
       </c>
-      <c r="G3" t="b">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="b">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>A stylish everyday Tote bag to carry your essentials, available in custom color in medium and large sizes</t>
         </is>
@@ -563,10 +574,11 @@
       <c r="F4" t="n">
         <v>700</v>
       </c>
-      <c r="G4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>An effortless style statement to complete your look</t>
         </is>
@@ -601,10 +613,15 @@
       <c r="F5" t="n">
         <v>1000</v>
       </c>
-      <c r="G5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Brown Model Clutch.jpeg</t>
+        </is>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>An effortless style statement to complete your look</t>
         </is>
@@ -639,10 +656,11 @@
       <c r="F6" t="n">
         <v>900</v>
       </c>
-      <c r="G6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>A timeless style statement with elegant handle</t>
         </is>
@@ -677,10 +695,15 @@
       <c r="F7" t="n">
         <v>1200</v>
       </c>
-      <c r="G7" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Blue Sling.jpeg</t>
+        </is>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>A timeless style statement with elegant handle</t>
         </is>
@@ -715,10 +738,11 @@
       <c r="F8" t="n">
         <v>1100</v>
       </c>
-      <c r="G8" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>A timeless style statement with elegant handle</t>
         </is>
@@ -753,10 +777,11 @@
       <c r="F9" t="n">
         <v>1400</v>
       </c>
-      <c r="G9" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>A timeless style statement with elegant handle</t>
         </is>
@@ -787,10 +812,11 @@
       <c r="F10" t="n">
         <v>650</v>
       </c>
-      <c r="G10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>Your everyday travel buddy, for that sturdy yet cute look</t>
         </is>
@@ -821,10 +847,15 @@
       <c r="F11" t="n">
         <v>850</v>
       </c>
-      <c r="G11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" t="inlineStr">
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Pink Baset.jpeg</t>
+        </is>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>Your everyday travel buddy, for that sturdy yet cute look</t>
         </is>
@@ -855,10 +886,11 @@
       <c r="F12" t="n">
         <v>1100</v>
       </c>
-      <c r="G12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H12" t="inlineStr">
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>Your everyday travel buddy, for that sturdy yet cute look</t>
         </is>
@@ -889,10 +921,11 @@
       <c r="F13" t="n">
         <v>750</v>
       </c>
-      <c r="G13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H13" t="inlineStr">
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
         </is>
@@ -923,10 +956,15 @@
       <c r="F14" t="n">
         <v>1000</v>
       </c>
-      <c r="G14" t="b">
-        <v>1</v>
-      </c>
-      <c r="H14" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Yellow Wooden Handle.jpeg</t>
+        </is>
+      </c>
+      <c r="H14" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
         </is>
@@ -957,10 +995,11 @@
       <c r="F15" t="n">
         <v>1400</v>
       </c>
-      <c r="G15" t="b">
-        <v>1</v>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="b">
+        <v>1</v>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
         </is>
@@ -991,10 +1030,11 @@
       <c r="F16" t="n">
         <v>750</v>
       </c>
-      <c r="G16" t="b">
-        <v>1</v>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="b">
+        <v>1</v>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
         </is>
@@ -1025,10 +1065,11 @@
       <c r="F17" t="n">
         <v>950</v>
       </c>
-      <c r="G17" t="b">
-        <v>1</v>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
         </is>
@@ -1059,10 +1100,11 @@
       <c r="F18" t="n">
         <v>850</v>
       </c>
-      <c r="G18" t="b">
-        <v>1</v>
-      </c>
-      <c r="H18" t="inlineStr">
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="b">
+        <v>1</v>
+      </c>
+      <c r="I18" t="inlineStr">
         <is>
           <t>Ultra stylish bag, a perfect head turner!</t>
         </is>
@@ -1093,10 +1135,15 @@
       <c r="F19" t="n">
         <v>1100</v>
       </c>
-      <c r="G19" t="b">
-        <v>1</v>
-      </c>
-      <c r="H19" t="inlineStr">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Eye Handle 1.jpeg, Eye Handle 2.png, Eye Handle 3.png, Dimensions Chart.png</t>
+        </is>
+      </c>
+      <c r="H19" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>Ultra stylish bag, a perfect head turner!</t>
         </is>
@@ -1127,10 +1174,11 @@
       <c r="F20" t="n">
         <v>1400</v>
       </c>
-      <c r="G20" t="b">
-        <v>1</v>
-      </c>
-      <c r="H20" t="inlineStr">
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="b">
+        <v>1</v>
+      </c>
+      <c r="I20" t="inlineStr">
         <is>
           <t>Ultra stylish bag, a perfect head turner!</t>
         </is>
@@ -1161,10 +1209,11 @@
       <c r="F21" t="n">
         <v>850</v>
       </c>
-      <c r="G21" t="b">
-        <v>1</v>
-      </c>
-      <c r="H21" t="inlineStr">
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
         </is>
@@ -1195,10 +1244,11 @@
       <c r="F22" t="n">
         <v>1000</v>
       </c>
-      <c r="G22" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" t="inlineStr">
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="b">
+        <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr">
         <is>
           <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
         </is>

</xml_diff>

<commit_message>
chore: nightly sync from Google Sheets [2026-03-09 09:40 UTC]
</commit_message>
<xml_diff>
--- a/data/Sheet1.xlsx
+++ b/data/Sheet1.xlsx
@@ -574,7 +574,11 @@
       <c r="F4" t="n">
         <v>700</v>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>/images/BrownModelClutch.jpeg</t>
+        </is>
+      </c>
       <c r="H4" t="b">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
chore: nightly sync from Google Sheets [2026-03-09 12:22 UTC]
</commit_message>
<xml_diff>
--- a/data/Sheet1.xlsx
+++ b/data/Sheet1.xlsx
@@ -574,11 +574,7 @@
       <c r="F4" t="n">
         <v>700</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>/images/BrownModelClutch.jpeg</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="b">
         <v>1</v>
       </c>
@@ -619,7 +615,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>/images/BrownModelClutch.jpeg</t>
+          <t>BrownModelClutch.jpeg</t>
         </is>
       </c>
       <c r="H5" t="b">

</xml_diff>

<commit_message>
chore: nightly sync from Google Sheets [2026-03-09 15:36 UTC]
</commit_message>
<xml_diff>
--- a/data/Sheet1.xlsx
+++ b/data/Sheet1.xlsx
@@ -712,7 +712,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BAG003</t>
+          <t>BAG004</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -751,7 +751,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BAG003</t>
+          <t>BAG004</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -790,7 +790,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BAG004</t>
+          <t>BAG005</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -825,7 +825,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BAG004</t>
+          <t>BAG005</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -864,7 +864,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BAG004</t>
+          <t>BAG005</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -899,7 +899,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG006</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -934,7 +934,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG006</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -973,7 +973,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG006</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1008,7 +1008,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG007</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1043,7 +1043,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG007</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1078,7 +1078,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG008</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1113,7 +1113,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG008</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1152,7 +1152,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG008</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BAG006</t>
+          <t>BAG009</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1222,7 +1222,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BAG006</t>
+          <t>BAG009</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">

</xml_diff>

<commit_message>
chore: nightly sync from Google Sheets [2026-03-24 03:45 UTC]
</commit_message>
<xml_diff>
--- a/data/Sheet1.xlsx
+++ b/data/Sheet1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="H2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -524,20 +524,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MULTI</t>
+          <t>Chocolate Brown</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1400</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
+        <v>1100</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>BrownTote.png, BrownTote1.png, BrownTote2.jpeg</t>
+        </is>
+      </c>
       <c r="H3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -548,22 +552,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BAG002</t>
+          <t>BAG001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Clutch Koodai</t>
+          <t>Tote Bag</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Clutch</t>
+          <t>Tote</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -572,15 +576,15 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>700</v>
+        <v>1400</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>An effortless style statement to complete your look</t>
+          <t>A stylish everyday Tote bag to carry your essentials, available in custom color in medium and large sizes</t>
         </is>
       </c>
     </row>
@@ -602,7 +606,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -611,13 +615,9 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>BrownModelClutch.jpeg</t>
-        </is>
-      </c>
+        <v>700</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="b">
         <v>1</v>
       </c>
@@ -630,22 +630,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BAG003</t>
+          <t>BAG002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sling with chain</t>
+          <t>Clutch Koodai</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sling</t>
+          <t>Clutch</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -654,15 +654,19 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>900</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
+        <v>1000</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>BrownModelClutch.jpeg</t>
+        </is>
+      </c>
       <c r="H6" t="b">
         <v>1</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>A timeless style statement with elegant handle</t>
+          <t>An effortless style statement to complete your look</t>
         </is>
       </c>
     </row>
@@ -684,7 +688,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -693,11 +697,11 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1200</v>
+        <v>900</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Blue Sling.jpeg</t>
+          <t>BlackWhite0.png, BlackWhite1.jpeg, BlackWhite2.jpeg</t>
         </is>
       </c>
       <c r="H7" t="b">
@@ -712,12 +716,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BAG004</t>
+          <t>BAG003</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sling with leather</t>
+          <t>Sling with chain</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -727,7 +731,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -736,9 +740,13 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
+        <v>1200</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>BlueSling.jpeg</t>
+        </is>
+      </c>
       <c r="H8" t="b">
         <v>1</v>
       </c>
@@ -766,7 +774,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -775,7 +783,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1400</v>
+        <v>1100</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="b">
@@ -790,35 +798,43 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG004</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Basket Koodai</t>
+          <t>Sling with leather</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Basket</t>
+          <t>Sling</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Blue White</t>
+        </is>
+      </c>
       <c r="F10" t="n">
-        <v>650</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
+        <v>1400</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>BlueWhiteSling0.png, BlueWhiteSling1.png, BlueWhiteSling2.jpeg, BlueWhiteSling3.jpeg</t>
+        </is>
+      </c>
       <c r="H10" t="b">
         <v>1</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
+          <t>A timeless style statement with elegant handle</t>
         </is>
       </c>
     </row>
@@ -840,18 +856,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>850</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Pink Basket.jpeg</t>
-        </is>
-      </c>
+        <v>650</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="b">
         <v>1</v>
       </c>
@@ -879,14 +891,18 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
+        <v>850</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PinkBasket0.png, PinkBasket01.png, PinkBasket.jpeg, PinkBasket1.png, </t>
+        </is>
+      </c>
       <c r="H12" t="b">
         <v>1</v>
       </c>
@@ -899,27 +915,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BAG006</t>
+          <t>BAG005</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Wooden handle Koodai</t>
+          <t>Basket Koodai</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Basket</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>10</v>
+        <v>1100</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="b">
@@ -927,7 +943,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
+          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
         </is>
       </c>
     </row>
@@ -949,18 +965,14 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Yellow Wooden Handle.jpeg</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="b">
         <v>1</v>
       </c>
@@ -988,14 +1000,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
       <c r="F15" t="n">
-        <v>1400</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
+        <v>1000</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>YellowWoodenHandle1.png, YellowWoodenHandle.jpeg</t>
+        </is>
+      </c>
       <c r="H15" t="b">
         <v>1</v>
       </c>
@@ -1008,12 +1028,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BAG007</t>
+          <t>BAG006</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Kai Koodai</t>
+          <t>Wooden handle Koodai</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1023,12 +1043,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>750</v>
+        <v>1400</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="b">
@@ -1036,7 +1056,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
+          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
         </is>
       </c>
     </row>
@@ -1058,12 +1078,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>950</v>
+        <v>750</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="b">
@@ -1078,12 +1098,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BAG008</t>
+          <t>BAG007</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Eye handle Koodai</t>
+          <t>Kai Koodai</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1093,12 +1113,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>850</v>
+        <v>950</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="b">
@@ -1106,7 +1126,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Ultra stylish bag, a perfect head turner!</t>
+          <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
         </is>
       </c>
     </row>
@@ -1128,16 +1148,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Dark Brown</t>
+        </is>
+      </c>
       <c r="F19" t="n">
-        <v>1100</v>
+        <v>850</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Eye Handle 1.jpeg, Eye Handle 2.png, Eye Handle 3.png, Dimensions Chart.png</t>
+          <t>Eye Handle 0.png</t>
         </is>
       </c>
       <c r="H19" t="b">
@@ -1167,14 +1191,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Dark Brown</t>
+        </is>
+      </c>
       <c r="F20" t="n">
-        <v>1400</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
+        <v>1100</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Eye Handle 1.jpeg, Eye Handle 2.png, Eye Handle 3.png, Dimensions Chart.png</t>
+        </is>
+      </c>
       <c r="H20" t="b">
         <v>1</v>
       </c>
@@ -1187,27 +1219,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BAG009</t>
+          <t>BAG008</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cute Pooja Koodai</t>
+          <t>Eye handle Koodai</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Wooden</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
-        <v>850</v>
+        <v>1400</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="b">
@@ -1215,7 +1247,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
+          <t>Ultra stylish bag, a perfect head turner!</t>
         </is>
       </c>
     </row>
@@ -1237,18 +1269,53 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>1000</v>
+        <v>850</v>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="b">
         <v>1</v>
       </c>
       <c r="I22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BAG009</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Cute Pooja Koodai</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" t="inlineStr">
         <is>
           <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
         </is>

</xml_diff>

<commit_message>
chore: nightly sync from Google Sheets [2026-03-25 03:56 UTC]
</commit_message>
<xml_diff>
--- a/data/Sheet1.xlsx
+++ b/data/Sheet1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,7 +486,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>MULTI</t>
+          <t>Chocolate Brown</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -494,7 +494,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Biscuit Knot Tote.jpg, White Tote Bag.jpg, Dimensions Chart.png</t>
+          <t>BrownTote.png, BrownTote1.png, BrownTote2.jpeg, Biscuit Knot Tote.jpg, White Tote Bag.jpg, Dimensions Chart.png</t>
         </is>
       </c>
       <c r="H2" t="b">
@@ -524,24 +524,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Chocolate Brown</t>
+          <t>MULTI</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>BrownTote.png, BrownTote1.png, BrownTote2.jpeg</t>
-        </is>
-      </c>
+        <v>1400</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -552,22 +548,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BAG001</t>
+          <t>BAG002</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tote Bag</t>
+          <t>Clutch Koodai</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tote</t>
+          <t>Clutch</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -576,15 +572,15 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1400</v>
+        <v>700</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>A stylish everyday Tote bag to carry your essentials, available in custom color in medium and large sizes</t>
+          <t>An effortless style statement to complete your look</t>
         </is>
       </c>
     </row>
@@ -606,7 +602,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -615,9 +611,13 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>700</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
+        <v>1000</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>BrownModelClutch.jpeg</t>
+        </is>
+      </c>
       <c r="H5" t="b">
         <v>1</v>
       </c>
@@ -630,17 +630,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BAG002</t>
+          <t>BAG004</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Clutch Koodai</t>
+          <t>Sling with leather</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Clutch</t>
+          <t>Sling</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -650,15 +650,15 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>MULTI</t>
+          <t>Blue White</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1000</v>
+        <v>1400</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>BrownModelClutch.jpeg</t>
+          <t>BlueWhiteSling1.png, BlueWhiteSling0.png, BlueWhiteSling2.jpeg, BlueWhiteSling3.jpeg</t>
         </is>
       </c>
       <c r="H6" t="b">
@@ -666,7 +666,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>An effortless style statement to complete your look</t>
+          <t>A timeless style statement with elegant handle</t>
         </is>
       </c>
     </row>
@@ -759,183 +759,179 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BAG004</t>
+          <t>BAG005</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Sling with leather</t>
+          <t>Basket Koodai</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sling</t>
+          <t>Basket</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>MULTI</t>
-        </is>
-      </c>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
+        <v>850</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PinkBasket0.png, PinkBasket01.png, PinkBasket.jpeg, PinkBasket1.png, </t>
+        </is>
+      </c>
       <c r="H9" t="b">
         <v>1</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>A timeless style statement with elegant handle</t>
+          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BAG004</t>
+          <t>BAG005</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sling with leather</t>
+          <t>Basket Koodai</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sling</t>
+          <t>Basket</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Blue White</t>
-        </is>
-      </c>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>1400</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>BlueWhiteSling0.png, BlueWhiteSling1.png, BlueWhiteSling2.jpeg, BlueWhiteSling3.jpeg</t>
-        </is>
-      </c>
+        <v>1100</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="b">
         <v>1</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>A timeless style statement with elegant handle</t>
+          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG006</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Basket Koodai</t>
+          <t>Wooden handle Koodai</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Basket</t>
+          <t>Wooden</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
       <c r="F11" t="n">
-        <v>650</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
+        <v>1000</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>YellowWoodenHandle1.png, YellowWoodenHandle.jpeg</t>
+        </is>
+      </c>
       <c r="H11" t="b">
         <v>1</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
+          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG006</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Basket Koodai</t>
+          <t>Wooden handle Koodai</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Basket</t>
+          <t>Wooden</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>850</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PinkBasket0.png, PinkBasket01.png, PinkBasket.jpeg, PinkBasket1.png, </t>
-        </is>
-      </c>
+        <v>1400</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="b">
         <v>1</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
+          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BAG005</t>
+          <t>BAG007</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Basket Koodai</t>
+          <t>Kai Koodai</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Basket</t>
+          <t>Wooden</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>1100</v>
+        <v>750</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="b">
@@ -943,19 +939,19 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Your everyday travel buddy, for that sturdy yet cute look</t>
+          <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BAG006</t>
+          <t>BAG007</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Wooden handle Koodai</t>
+          <t>Kai Koodai</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -965,12 +961,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>10</v>
+        <v>950</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="b">
@@ -978,19 +974,19 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
+          <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BAG006</t>
+          <t>BAG008</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Wooden handle Koodai</t>
+          <t>Eye handle Koodai</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1000,20 +996,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Yellow</t>
+          <t>Dark Brown</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1000</v>
+        <v>850</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>YellowWoodenHandle1.png, YellowWoodenHandle.jpeg</t>
+          <t>Eye Handle 0.png</t>
         </is>
       </c>
       <c r="H15" t="b">
@@ -1021,19 +1017,19 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
+          <t>Ultra stylish bag, a perfect head turner!</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BAG006</t>
+          <t>BAG008</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Wooden handle Koodai</t>
+          <t>Eye handle Koodai</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1043,32 +1039,40 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Dark Brown</t>
+        </is>
+      </c>
       <c r="F16" t="n">
-        <v>1400</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
+        <v>1100</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Eye Handle 1.jpeg, Eye Handle 2.png, Eye Handle 3.png, Dimensions Chart.png</t>
+        </is>
+      </c>
       <c r="H16" t="b">
         <v>1</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Comfort and elegance woven into a bag, comes in custom sizes and colours of your choice!</t>
+          <t>Ultra stylish bag, a perfect head turner!</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BAG007</t>
+          <t>BAG008</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Kai Koodai</t>
+          <t>Eye handle Koodai</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1078,12 +1082,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>750</v>
+        <v>1400</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="b">
@@ -1091,34 +1095,34 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
+          <t>Ultra stylish bag, a perfect head turner!</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BAG007</t>
+          <t>BAG009</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Kai Koodai</t>
+          <t>Cute Pooja Koodai</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>950</v>
+        <v>850</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="b">
@@ -1126,196 +1130,40 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>The show stopping bag that can redefine your fashion while providing space for that extra shopping!</t>
+          <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BAG008</t>
+          <t>BAG009</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Eye handle Koodai</t>
+          <t>Cute Pooja Koodai</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Wooden</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Dark Brown</t>
-        </is>
-      </c>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>850</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Eye Handle 0.png</t>
-        </is>
-      </c>
+        <v>1000</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="b">
         <v>1</v>
       </c>
       <c r="I19" t="inlineStr">
-        <is>
-          <t>Ultra stylish bag, a perfect head turner!</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>BAG008</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Eye handle Koodai</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Wooden</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Dark Brown</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>1100</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Eye Handle 1.jpeg, Eye Handle 2.png, Eye Handle 3.png, Dimensions Chart.png</t>
-        </is>
-      </c>
-      <c r="H20" t="b">
-        <v>1</v>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Ultra stylish bag, a perfect head turner!</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>BAG008</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Eye handle Koodai</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Wooden</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="n">
-        <v>1400</v>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="b">
-        <v>1</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Ultra stylish bag, a perfect head turner!</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>BAG009</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Cute Pooja Koodai</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Others</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="n">
-        <v>850</v>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="b">
-        <v>1</v>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>BAG009</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Cute Pooja Koodai</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Others</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="b">
-        <v>1</v>
-      </c>
-      <c r="I23" t="inlineStr">
         <is>
           <t xml:space="preserve">The right bag for those days you wish to be extra charming </t>
         </is>

</xml_diff>

<commit_message>
chore: nightly sync from Google Sheets [2026-04-12 04:23 UTC]
</commit_message>
<xml_diff>
--- a/data/Sheet1.xlsx
+++ b/data/Sheet1.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>BrownTote.png, BrownTote1.png, BrownTote2.jpeg, Biscuit Knot Tote.jpg, White Tote Bag.jpg, Dimensions Chart.png</t>
+          <t>BrownTote2.jpeg, BrownTote.png, Biscuit Knot Tote.jpg, White Tote Bag.jpg, Dimensions Chart.png</t>
         </is>
       </c>
       <c r="H2" t="b">
@@ -658,7 +658,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>BlueWhiteSling1.png, BlueWhiteSling0.png, BlueWhiteSling2.jpeg, BlueWhiteSling3.jpeg</t>
+          <t xml:space="preserve">BlueWhiteSling3.jpeg, BlueWhiteSling1.png, BlueWhiteSling0.png, BlueWhiteSling2.jpeg, </t>
         </is>
       </c>
       <c r="H6" t="b">
@@ -701,7 +701,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>BlackWhite0.png, BlackWhite1.jpeg, BlackWhite2.jpeg</t>
+          <t xml:space="preserve"> BlackWhite1.jpeg, BlackWhite0.png, BlackWhite2.jpeg</t>
         </is>
       </c>
       <c r="H7" t="b">

</xml_diff>